<commit_message>
boys x < 1e-15
</commit_message>
<xml_diff>
--- a/Coulomb_matrix.xlsx
+++ b/Coulomb_matrix.xlsx
@@ -418,13 +418,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>17.72500617342665</v>
+        <v>13.72845922179257</v>
       </c>
       <c r="B1" t="n">
-        <v>3.661131345875514</v>
+        <v>2.425481114663914</v>
       </c>
       <c r="C1" t="n">
-        <v>2.71706969423415</v>
+        <v>1.901804951241529</v>
       </c>
       <c r="D1" t="n">
         <v>0</v>
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="F1" t="n">
-        <v>0.4486701413504272</v>
+        <v>0.05278350465146915</v>
       </c>
       <c r="G1" t="n">
         <v>0</v>
@@ -442,16 +442,16 @@
         <v>0</v>
       </c>
       <c r="I1" t="n">
-        <v>0.05948364228025752</v>
+        <v>0.007210271412172451</v>
       </c>
       <c r="J1" t="n">
-        <v>1.519420907240848e-24</v>
+        <v>6.468932386619966e-25</v>
       </c>
       <c r="K1" t="n">
-        <v>2.607981505652781e-07</v>
+        <v>1.535841145562214e-07</v>
       </c>
       <c r="L1" t="n">
-        <v>0.01692914605411481</v>
+        <v>0.01225140799400638</v>
       </c>
       <c r="M1" t="n">
         <v>0</v>
@@ -460,7 +460,7 @@
         <v>0</v>
       </c>
       <c r="O1" t="n">
-        <v>-1.028198032478294e-06</v>
+        <v>-7.614647360752392e-07</v>
       </c>
       <c r="P1" t="n">
         <v>0</v>
@@ -469,16 +469,16 @@
         <v>0</v>
       </c>
       <c r="R1" t="n">
-        <v>-0.07033513946566122</v>
+        <v>-0.05427125527045636</v>
       </c>
       <c r="S1" t="n">
-        <v>9.856531882326483e-05</v>
+        <v>5.674603015228227e-05</v>
       </c>
       <c r="T1" t="n">
-        <v>0.41028017528847</v>
+        <v>0.2974519856972697</v>
       </c>
       <c r="U1" t="n">
-        <v>0.8658396667432683</v>
+        <v>0.6123341462429266</v>
       </c>
       <c r="V1" t="n">
         <v>0</v>
@@ -487,7 +487,7 @@
         <v>0</v>
       </c>
       <c r="X1" t="n">
-        <v>-0.7715763974044589</v>
+        <v>-0.599797732256183</v>
       </c>
       <c r="Y1" t="n">
         <v>0</v>
@@ -496,18 +496,18 @@
         <v>0</v>
       </c>
       <c r="AA1" t="n">
-        <v>-1.409831173295371</v>
+        <v>-1.082744751304861</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3.661131345875514</v>
+        <v>2.425481114663914</v>
       </c>
       <c r="B2" t="n">
-        <v>11.7953387318627</v>
+        <v>7.367972089520421</v>
       </c>
       <c r="C2" t="n">
-        <v>8.057331094449143</v>
+        <v>5.153824876435855</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -516,7 +516,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>3.470722540705811</v>
+        <v>0.3345861651149042</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -525,16 +525,16 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1.620692613473578</v>
+        <v>0.2075005320679499</v>
       </c>
       <c r="J2" t="n">
-        <v>2.66504237768089e-07</v>
+        <v>1.535841145562213e-07</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0009858939824930924</v>
+        <v>0.0004834622632400072</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1156499529615993</v>
+        <v>0.08661652229379095</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>-0.004556953322077898</v>
+        <v>-0.001374558280326941</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -552,16 +552,16 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.09064878628384998</v>
+        <v>-0.313054428907012</v>
       </c>
       <c r="S2" t="n">
-        <v>0.113432854820305</v>
+        <v>0.08385217855767998</v>
       </c>
       <c r="T2" t="n">
-        <v>2.455316568081653</v>
+        <v>1.367532737419496</v>
       </c>
       <c r="U2" t="n">
-        <v>3.207219792326001</v>
+        <v>2.055018502891799</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>-1.931475448214684</v>
+        <v>-2.16760635751014</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -579,18 +579,18 @@
         <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>-3.887214466383659</v>
+        <v>-3.146205412947956</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2.71706969423415</v>
+        <v>1.901804951241529</v>
       </c>
       <c r="B3" t="n">
-        <v>8.057331094449143</v>
+        <v>5.153824876435855</v>
       </c>
       <c r="C3" t="n">
-        <v>8.549601478812308</v>
+        <v>5.431862159025142</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -599,7 +599,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>2.448048533434815</v>
+        <v>0.3095571448914275</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -608,16 +608,16 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>3.188150954447806</v>
+        <v>0.5075252945013249</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01672729881038509</v>
+        <v>0.01225140799400637</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1089987412453257</v>
+        <v>0.08661652229379094</v>
       </c>
       <c r="L3" t="n">
-        <v>1.025515637774102</v>
+        <v>0.4025291001427244</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -626,7 +626,7 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.007383933264485859</v>
+        <v>-0.1129430858418718</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -635,16 +635,16 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>-2.941037486242763</v>
+        <v>-0.9170028130182086</v>
       </c>
       <c r="S3" t="n">
-        <v>0.7694354589371539</v>
+        <v>0.5514055018286396</v>
       </c>
       <c r="T3" t="n">
-        <v>3.281542563816319</v>
+        <v>2.339182697798996</v>
       </c>
       <c r="U3" t="n">
-        <v>3.324992764035244</v>
+        <v>3.075874547195067</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -653,7 +653,7 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>-3.86868701613897</v>
+        <v>-2.169268185931883</v>
       </c>
       <c r="Y3" t="n">
         <v>0</v>
@@ -662,7 +662,7 @@
         <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>-3.982228449644786</v>
+        <v>-3.398737595875454</v>
       </c>
     </row>
     <row r="4">
@@ -676,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>12.2402806654926</v>
+        <v>8.274748504302968</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -685,7 +685,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4.809969513216682</v>
+        <v>3.341260378228474</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -703,7 +703,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0009956030670435325</v>
+        <v>0.0001782133990677275</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -712,7 +712,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.01856356769511494</v>
+        <v>0.0477181031060863</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>-0.1146799619616365</v>
+        <v>0.7023258820844938</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>-2.45635663933435</v>
+        <v>1.080208234691793</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
@@ -762,7 +762,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>12.26235431208335</v>
+        <v>8.296934678791304</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -771,7 +771,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>4.861208802228177</v>
+        <v>3.41550398576649</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -789,7 +789,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.000996956682445471</v>
+        <v>0.0001785015305702519</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -798,7 +798,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.01804364116715514</v>
+        <v>0.04848551154802327</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -816,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>-0.106923431438434</v>
+        <v>0.7113861977620545</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
@@ -825,7 +825,7 @@
         <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>-2.439483664451092</v>
+        <v>1.104996748025871</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
@@ -833,13 +833,13 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.4486701413504272</v>
+        <v>0.05278350465146915</v>
       </c>
       <c r="B6" t="n">
-        <v>3.470722540705811</v>
+        <v>0.3345861651149042</v>
       </c>
       <c r="C6" t="n">
-        <v>2.448048533434815</v>
+        <v>0.3095571448914275</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>12.53618899178513</v>
+        <v>8.436988790762461</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -857,16 +857,16 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>5.483038668120161</v>
+        <v>3.570980524318417</v>
       </c>
       <c r="J6" t="n">
-        <v>9.148697745882016e-07</v>
+        <v>7.609274310020573e-07</v>
       </c>
       <c r="K6" t="n">
-        <v>0.004692057677492125</v>
+        <v>0.001368697708389186</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.007001023411008306</v>
+        <v>0.1114209406848399</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -875,7 +875,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.01937528949908188</v>
+        <v>-0.003696700192926637</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -884,16 +884,16 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0.09763683198495104</v>
+        <v>-0.355573871190547</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4400283982304294</v>
+        <v>0.1936684732668824</v>
       </c>
       <c r="T6" t="n">
-        <v>2.1055102714432</v>
+        <v>1.494159329061754</v>
       </c>
       <c r="U6" t="n">
-        <v>2.673103201184555</v>
+        <v>1.023943964186715</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
@@ -902,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.8237603665705511</v>
+        <v>-1.941206507651286</v>
       </c>
       <c r="Y6" t="n">
         <v>0</v>
@@ -911,7 +911,7 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.8084629721561751</v>
+        <v>-0.4240457302122232</v>
       </c>
     </row>
     <row r="7">
@@ -925,7 +925,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>4.809969513216682</v>
+        <v>3.341260378228474</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -934,7 +934,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>-10.92820993404806</v>
+        <v>5.184508432734076</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -952,7 +952,7 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.02312083321483989</v>
+        <v>0.04462874363360245</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -961,7 +961,7 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0.653453995998958</v>
+        <v>0.3500267147882509</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -979,7 +979,7 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>4.692079266861452</v>
+        <v>1.668529833194776</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.661611796948493</v>
+        <v>2.773294132000843</v>
       </c>
       <c r="Z7" t="n">
         <v>0</v>
@@ -1011,7 +1011,7 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>4.861208802228177</v>
+        <v>3.41550398576649</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>-10.91319874490682</v>
+        <v>5.184409717898171</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.02296968487951888</v>
+        <v>0.04462938943735213</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1047,7 +1047,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.6546948860037229</v>
+        <v>0.3499981105401278</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1065,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>4.691567316273273</v>
+        <v>1.668428995917327</v>
       </c>
       <c r="X8" t="n">
         <v>0</v>
@@ -1074,7 +1074,7 @@
         <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>5.664332984950206</v>
+        <v>2.773264146949486</v>
       </c>
       <c r="AA8" t="n">
         <v>0</v>
@@ -1082,13 +1082,13 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.05948364228025752</v>
+        <v>0.007210271412172451</v>
       </c>
       <c r="B9" t="n">
-        <v>1.620692613473578</v>
+        <v>0.2075005320679499</v>
       </c>
       <c r="C9" t="n">
-        <v>3.188150954447806</v>
+        <v>0.5075252945013249</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1097,7 +1097,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5.483038668120161</v>
+        <v>3.570980524318417</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1106,16 +1106,16 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>-13.54916293710976</v>
+        <v>5.520104838796613</v>
       </c>
       <c r="J9" t="n">
-        <v>0.07123205430148202</v>
+        <v>0.05425021485936828</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.06267817501791145</v>
+        <v>0.3127150200107867</v>
       </c>
       <c r="L9" t="n">
-        <v>3.017338689096679</v>
+        <v>0.9149335269915267</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0.141964855980248</v>
+        <v>-0.3657547104789904</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -1133,16 +1133,16 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>-3.201762054718563</v>
+        <v>-1.635621923267868</v>
       </c>
       <c r="S9" t="n">
-        <v>3.392583943633511</v>
+        <v>1.186719368286791</v>
       </c>
       <c r="T9" t="n">
-        <v>7.128283302631091</v>
+        <v>3.322748390595217</v>
       </c>
       <c r="U9" t="n">
-        <v>6.04688196478084</v>
+        <v>2.701091179632882</v>
       </c>
       <c r="V9" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>-2.41603817331059</v>
+        <v>-1.313923727158325</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
@@ -1160,18 +1160,18 @@
         <v>0</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.9628671033800138</v>
+        <v>0.1989722918107112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.519420907240848e-24</v>
+        <v>6.468932386619966e-25</v>
       </c>
       <c r="B10" t="n">
-        <v>2.66504237768089e-07</v>
+        <v>1.535841145562213e-07</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01672729881038509</v>
+        <v>0.01225140799400637</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1180,7 +1180,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>9.148697745882016e-07</v>
+        <v>7.609274310020573e-07</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1189,16 +1189,16 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0.07123205430148202</v>
+        <v>0.05425021485936828</v>
       </c>
       <c r="J10" t="n">
-        <v>17.96610250914503</v>
+        <v>13.72178781226155</v>
       </c>
       <c r="K10" t="n">
-        <v>3.65973802164041</v>
+        <v>2.423914845583349</v>
       </c>
       <c r="L10" t="n">
-        <v>2.727874650419917</v>
+        <v>1.90068533861091</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
@@ -1207,7 +1207,7 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>-0.3454947072788586</v>
+        <v>-0.0519595639822607</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1216,16 +1216,16 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.04607555509673834</v>
+        <v>-0.007096852975960076</v>
       </c>
       <c r="S10" t="n">
-        <v>9.618400358081792e-05</v>
+        <v>5.666047666247473e-05</v>
       </c>
       <c r="T10" t="n">
-        <v>0.4029374356004369</v>
+        <v>0.2972556811508809</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8539117079926567</v>
+        <v>0.6119602248322812</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>0.7784855997092419</v>
+        <v>0.5994239514891161</v>
       </c>
       <c r="Y10" t="n">
         <v>0</v>
@@ -1243,18 +1243,18 @@
         <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.40567882475756</v>
+        <v>1.082116365985503</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2.607981505652781e-07</v>
+        <v>1.535841145562214e-07</v>
       </c>
       <c r="B11" t="n">
-        <v>0.0009858939824930924</v>
+        <v>0.0004834622632400072</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1089987412453257</v>
+        <v>0.08661652229379094</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -1263,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.004692057677492125</v>
+        <v>0.001368697708389186</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -1272,16 +1272,16 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.06267817501791145</v>
+        <v>0.3127150200107867</v>
       </c>
       <c r="J11" t="n">
-        <v>3.65973802164041</v>
+        <v>2.423914845583349</v>
       </c>
       <c r="K11" t="n">
-        <v>11.45679063950046</v>
+        <v>7.361240198480571</v>
       </c>
       <c r="L11" t="n">
-        <v>7.888051147919526</v>
+        <v>5.148698929850372</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>-2.974910982132009</v>
+        <v>-0.3290864764165811</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1299,16 +1299,16 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>-1.489233995184495</v>
+        <v>-0.2039882654453667</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1214214831590169</v>
+        <v>0.08345480494086495</v>
       </c>
       <c r="T11" t="n">
-        <v>2.580874281046059</v>
+        <v>1.365121945825865</v>
       </c>
       <c r="U11" t="n">
-        <v>3.205463752175854</v>
+        <v>2.052383413121853</v>
       </c>
       <c r="V11" t="n">
         <v>0</v>
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>1.861880087016957</v>
+        <v>2.165188707887395</v>
       </c>
       <c r="Y11" t="n">
         <v>0</v>
@@ -1326,18 +1326,18 @@
         <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>3.660787614650573</v>
+        <v>3.143762882042221</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.01692914605411481</v>
+        <v>0.01225140799400638</v>
       </c>
       <c r="B12" t="n">
-        <v>0.1156499529615993</v>
+        <v>0.08661652229379095</v>
       </c>
       <c r="C12" t="n">
-        <v>1.025515637774102</v>
+        <v>0.4025291001427244</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -1346,7 +1346,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.007001023411008306</v>
+        <v>0.1114209406848399</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -1355,16 +1355,16 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>3.017338689096679</v>
+        <v>0.9149335269915267</v>
       </c>
       <c r="J12" t="n">
-        <v>2.727874650419917</v>
+        <v>1.90068533861091</v>
       </c>
       <c r="K12" t="n">
-        <v>7.888051147919526</v>
+        <v>5.148698929850372</v>
       </c>
       <c r="L12" t="n">
-        <v>8.580977827401467</v>
+        <v>5.425316385251865</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -1373,7 +1373,7 @@
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>-2.206191083916387</v>
+        <v>-0.3043637339652328</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -1382,16 +1382,16 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>-1.65446123821265</v>
+        <v>-0.4987128994133594</v>
       </c>
       <c r="S12" t="n">
-        <v>0.7776575318418943</v>
+        <v>0.5480044009982044</v>
       </c>
       <c r="T12" t="n">
-        <v>3.106597251060878</v>
+        <v>2.331222438032529</v>
       </c>
       <c r="U12" t="n">
-        <v>3.148213782455421</v>
+        <v>3.069076321864357</v>
       </c>
       <c r="V12" t="n">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>4.268720005111021</v>
+        <v>2.171946915734052</v>
       </c>
       <c r="Y12" t="n">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>4.283930900581249</v>
+        <v>3.399704775832141</v>
       </c>
     </row>
     <row r="13">
@@ -1423,7 +1423,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0009956030670435325</v>
+        <v>0.0001782133990677275</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -1432,7 +1432,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.02312083321483989</v>
+        <v>0.04462874363360245</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1450,7 +1450,7 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>13.01854990724892</v>
+        <v>8.278399703876518</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1459,7 +1459,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>4.199683224909266</v>
+        <v>3.348473142471157</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -1477,7 +1477,7 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>-0.2058046097653452</v>
+        <v>0.7044243605331411</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
@@ -1486,7 +1486,7 @@
         <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>-2.543867914054363</v>
+        <v>1.083664569831226</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -1509,7 +1509,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0.000996956682445471</v>
+        <v>0.0001785015305702519</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1518,7 +1518,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.02296968487951888</v>
+        <v>0.04462938943735213</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1536,7 +1536,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>13.0668474846394</v>
+        <v>8.300536879068691</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -1545,7 +1545,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.226954717789074</v>
+        <v>3.422715626940646</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1563,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.2015879526508015</v>
+        <v>0.7134823622163563</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>-2.535054021863906</v>
+        <v>1.108453806498179</v>
       </c>
       <c r="AA14" t="n">
         <v>0</v>
@@ -1580,13 +1580,13 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-1.028198032478294e-06</v>
+        <v>-7.614647360752392e-07</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.004556953322077898</v>
+        <v>-0.001374558280326941</v>
       </c>
       <c r="C15" t="n">
-        <v>0.007383933264485859</v>
+        <v>-0.1129430858418718</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -1595,7 +1595,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.01937528949908188</v>
+        <v>-0.003696700192926637</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -1604,16 +1604,16 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0.141964855980248</v>
+        <v>-0.3657547104789904</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.3454947072788586</v>
+        <v>-0.0519595639822607</v>
       </c>
       <c r="K15" t="n">
-        <v>-2.974910982132009</v>
+        <v>-0.3290864764165811</v>
       </c>
       <c r="L15" t="n">
-        <v>-2.206191083916387</v>
+        <v>-0.3043637339652328</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>13.42617720932543</v>
+        <v>8.441525057790935</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
@@ -1631,16 +1631,16 @@
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>4.49718070998838</v>
+        <v>3.579194678288036</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.4248479668265994</v>
+        <v>-0.1926461722131549</v>
       </c>
       <c r="T15" t="n">
-        <v>-1.667560383824083</v>
+        <v>-1.489476111077466</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.95044565406208</v>
+        <v>-1.019827472314353</v>
       </c>
       <c r="V15" t="n">
         <v>0</v>
@@ -1649,7 +1649,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>-0.4577697028973169</v>
+        <v>-1.931856534611696</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -1658,7 +1658,7 @@
         <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.279939865673288</v>
+        <v>-0.4143579642504828</v>
       </c>
     </row>
     <row r="16">
@@ -1672,7 +1672,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.01856356769511494</v>
+        <v>0.0477181031060863</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1681,7 +1681,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0.653453995998958</v>
+        <v>0.3500267147882509</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1699,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>4.199683224909266</v>
+        <v>3.348473142471157</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>-11.7648755060484</v>
+        <v>5.231356395868163</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
@@ -1726,7 +1726,7 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>4.644478927122703</v>
+        <v>1.696998376714411</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
@@ -1735,7 +1735,7 @@
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>5.479396668133068</v>
+        <v>2.835618098571434</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.01804364116715514</v>
+        <v>0.04848551154802327</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1767,7 +1767,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6546948860037229</v>
+        <v>0.3499981105401278</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1785,7 +1785,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>4.226954717789074</v>
+        <v>3.422715626940646</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -1794,7 +1794,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>-11.76121995407672</v>
+        <v>5.231264699201519</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -1812,7 +1812,7 @@
         <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>4.637736688581933</v>
+        <v>1.696931568621135</v>
       </c>
       <c r="X17" t="n">
         <v>0</v>
@@ -1821,7 +1821,7 @@
         <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>5.482191757330714</v>
+        <v>2.835582125834184</v>
       </c>
       <c r="AA17" t="n">
         <v>0</v>
@@ -1829,13 +1829,13 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>-0.07033513946566122</v>
+        <v>-0.05427125527045636</v>
       </c>
       <c r="B18" t="n">
-        <v>0.09064878628384998</v>
+        <v>-0.313054428907012</v>
       </c>
       <c r="C18" t="n">
-        <v>-2.941037486242763</v>
+        <v>-0.9170028130182086</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.09763683198495104</v>
+        <v>-0.355573871190547</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1853,16 +1853,16 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>-3.201762054718563</v>
+        <v>-1.635621923267868</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.04607555509673834</v>
+        <v>-0.007096852975960076</v>
       </c>
       <c r="K18" t="n">
-        <v>-1.489233995184495</v>
+        <v>-0.2039882654453667</v>
       </c>
       <c r="L18" t="n">
-        <v>-1.65446123821265</v>
+        <v>-0.4987128994133594</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>4.49718070998838</v>
+        <v>3.579194678288036</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1880,16 +1880,16 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>-14.02182322272287</v>
+        <v>5.570663803899585</v>
       </c>
       <c r="S18" t="n">
-        <v>-3.288790884200119</v>
+        <v>-1.178989985987841</v>
       </c>
       <c r="T18" t="n">
-        <v>-4.687658316320815</v>
+        <v>-3.303073275551746</v>
       </c>
       <c r="U18" t="n">
-        <v>-3.68952740972431</v>
+        <v>-2.684745117313242</v>
       </c>
       <c r="V18" t="n">
         <v>0</v>
@@ -1898,7 +1898,7 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>-2.59282293431329</v>
+        <v>-1.282498459067561</v>
       </c>
       <c r="Y18" t="n">
         <v>0</v>
@@ -1907,18 +1907,18 @@
         <v>0</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.4547387423596508</v>
+        <v>0.2741241008832271</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>9.856531882326483e-05</v>
+        <v>5.674603015228227e-05</v>
       </c>
       <c r="B19" t="n">
-        <v>0.113432854820305</v>
+        <v>0.08385217855767998</v>
       </c>
       <c r="C19" t="n">
-        <v>0.7694354589371539</v>
+        <v>0.5514055018286396</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.4400283982304294</v>
+        <v>0.1936684732668824</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1936,16 +1936,16 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>3.392583943633511</v>
+        <v>1.186719368286791</v>
       </c>
       <c r="J19" t="n">
-        <v>9.618400358081792e-05</v>
+        <v>5.666047666247473e-05</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1214214831590169</v>
+        <v>0.08345480494086495</v>
       </c>
       <c r="L19" t="n">
-        <v>0.7776575318418943</v>
+        <v>0.5480044009982044</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
@@ -1954,7 +1954,7 @@
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>-0.4248479668265994</v>
+        <v>-0.1926461722131549</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -1963,16 +1963,16 @@
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>-3.288790884200119</v>
+        <v>-1.178989985987841</v>
       </c>
       <c r="S19" t="n">
-        <v>10.44993671202419</v>
+        <v>8.536468144470549</v>
       </c>
       <c r="T19" t="n">
-        <v>3.224839781135127</v>
+        <v>1.471756295915991</v>
       </c>
       <c r="U19" t="n">
-        <v>2.381962147400184</v>
+        <v>1.346306166324287</v>
       </c>
       <c r="V19" t="n">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         <v>0</v>
       </c>
       <c r="X19" t="n">
-        <v>0.3757895524307646</v>
+        <v>4.83554168928535e-17</v>
       </c>
       <c r="Y19" t="n">
         <v>0</v>
@@ -1990,18 +1990,18 @@
         <v>0</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.05992407407311829</v>
+        <v>1.430469241323062e-17</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.41028017528847</v>
+        <v>0.2974519856972697</v>
       </c>
       <c r="B20" t="n">
-        <v>2.455316568081653</v>
+        <v>1.367532737419496</v>
       </c>
       <c r="C20" t="n">
-        <v>3.281542563816319</v>
+        <v>2.339182697798996</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -2010,7 +2010,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>2.1055102714432</v>
+        <v>1.494159329061754</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -2019,16 +2019,16 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>7.128283302631091</v>
+        <v>3.322748390595217</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4029374356004369</v>
+        <v>0.2972556811508809</v>
       </c>
       <c r="K20" t="n">
-        <v>2.580874281046059</v>
+        <v>1.365121945825865</v>
       </c>
       <c r="L20" t="n">
-        <v>3.106597251060878</v>
+        <v>2.331222438032529</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>-1.667560383824083</v>
+        <v>-1.489476111077466</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -2046,16 +2046,16 @@
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>-4.687658316320815</v>
+        <v>-3.303073275551746</v>
       </c>
       <c r="S20" t="n">
-        <v>3.224839781135127</v>
+        <v>1.471756295915991</v>
       </c>
       <c r="T20" t="n">
-        <v>7.989897634820727</v>
+        <v>5.641945890180879</v>
       </c>
       <c r="U20" t="n">
-        <v>9.096464386556885</v>
+        <v>4.4183917809787</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
@@ -2064,7 +2064,7 @@
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>1.081501320590609</v>
+        <v>6.507381439257998e-16</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -2073,18 +2073,18 @@
         <v>0</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.2488233324784572</v>
+        <v>5.975038172567615e-16</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.8658396667432683</v>
+        <v>0.6123341462429266</v>
       </c>
       <c r="B21" t="n">
-        <v>3.207219792326001</v>
+        <v>2.055018502891799</v>
       </c>
       <c r="C21" t="n">
-        <v>3.324992764035244</v>
+        <v>3.075874547195067</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -2093,7 +2093,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2.673103201184555</v>
+        <v>1.023943964186715</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -2102,16 +2102,16 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>6.04688196478084</v>
+        <v>2.701091179632882</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8539117079926567</v>
+        <v>0.6119602248322812</v>
       </c>
       <c r="K21" t="n">
-        <v>3.205463752175854</v>
+        <v>2.052383413121853</v>
       </c>
       <c r="L21" t="n">
-        <v>3.148213782455421</v>
+        <v>3.069076321864357</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -2120,7 +2120,7 @@
         <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>-1.95044565406208</v>
+        <v>-1.019827472314353</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -2129,16 +2129,16 @@
         <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>-3.68952740972431</v>
+        <v>-2.684745117313242</v>
       </c>
       <c r="S21" t="n">
-        <v>2.381962147400184</v>
+        <v>1.346306166324287</v>
       </c>
       <c r="T21" t="n">
-        <v>9.096464386556885</v>
+        <v>4.4183917809787</v>
       </c>
       <c r="U21" t="n">
-        <v>9.139286797251835</v>
+        <v>4.874123452564334</v>
       </c>
       <c r="V21" t="n">
         <v>0</v>
@@ -2147,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>0.5912943022102487</v>
+        <v>1.747733902046633e-16</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.4538947839540482</v>
+        <v>9.033572501149223e-16</v>
       </c>
     </row>
     <row r="22">
@@ -2170,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1146799619616365</v>
+        <v>0.7023258820844938</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -2179,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>4.692079266861452</v>
+        <v>1.668529833194776</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -2197,7 +2197,7 @@
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>-0.2058046097653452</v>
+        <v>0.7044243605331411</v>
       </c>
       <c r="N22" t="n">
         <v>0</v>
@@ -2206,7 +2206,7 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>4.644478927122703</v>
+        <v>1.696998376714411</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -2224,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>33.59570791180811</v>
+        <v>6.185197598246612</v>
       </c>
       <c r="W22" t="n">
         <v>0</v>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="Y22" t="n">
-        <v>5.777224364122791</v>
+        <v>3.186199056322138</v>
       </c>
       <c r="Z22" t="n">
         <v>0</v>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.106923431438434</v>
+        <v>0.7113861977620545</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -2265,7 +2265,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4.691567316273273</v>
+        <v>1.668428995917327</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -2283,7 +2283,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>-0.2015879526508015</v>
+        <v>0.7134823622163563</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -2292,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.637736688581933</v>
+        <v>1.696931568621135</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2310,7 +2310,7 @@
         <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>33.6155046985315</v>
+        <v>6.184183450856056</v>
       </c>
       <c r="X23" t="n">
         <v>0</v>
@@ -2319,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="Z23" t="n">
-        <v>5.800013154550886</v>
+        <v>3.186849911762807</v>
       </c>
       <c r="AA23" t="n">
         <v>0</v>
@@ -2327,13 +2327,13 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>-0.7715763974044589</v>
+        <v>-0.599797732256183</v>
       </c>
       <c r="B24" t="n">
-        <v>-1.931475448214684</v>
+        <v>-2.16760635751014</v>
       </c>
       <c r="C24" t="n">
-        <v>-3.86868701613897</v>
+        <v>-2.169268185931883</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.8237603665705511</v>
+        <v>-1.941206507651286</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -2351,16 +2351,16 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>-2.41603817331059</v>
+        <v>-1.313923727158325</v>
       </c>
       <c r="J24" t="n">
-        <v>0.7784855997092419</v>
+        <v>0.5994239514891161</v>
       </c>
       <c r="K24" t="n">
-        <v>1.861880087016957</v>
+        <v>2.165188707887395</v>
       </c>
       <c r="L24" t="n">
-        <v>4.268720005111021</v>
+        <v>2.171946915734052</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
@@ -2369,7 +2369,7 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>-0.4577697028973169</v>
+        <v>-1.931856534611696</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -2378,16 +2378,16 @@
         <v>0</v>
       </c>
       <c r="R24" t="n">
-        <v>-2.59282293431329</v>
+        <v>-1.282498459067561</v>
       </c>
       <c r="S24" t="n">
-        <v>0.3757895524307646</v>
+        <v>4.83554168928535e-17</v>
       </c>
       <c r="T24" t="n">
-        <v>1.081501320590609</v>
+        <v>6.507381439257998e-16</v>
       </c>
       <c r="U24" t="n">
-        <v>0.5912943022102487</v>
+        <v>1.747733902046633e-16</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -2396,7 +2396,7 @@
         <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>40.10692237067642</v>
+        <v>6.945292341573849</v>
       </c>
       <c r="Y24" t="n">
         <v>0</v>
@@ -2405,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="AA24" t="n">
-        <v>7.400257187162005</v>
+        <v>3.83372519930778</v>
       </c>
     </row>
     <row r="25">
@@ -2419,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>-2.45635663933435</v>
+        <v>1.080208234691793</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>5.661611796948493</v>
+        <v>2.773294132000843</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -2446,7 +2446,7 @@
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>-2.543867914054363</v>
+        <v>1.083664569831226</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2455,7 +2455,7 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>5.479396668133068</v>
+        <v>2.835618098571434</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
@@ -2473,7 +2473,7 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>5.777224364122791</v>
+        <v>3.186199056322138</v>
       </c>
       <c r="W25" t="n">
         <v>0</v>
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>6.104390756662324</v>
+        <v>4.852972916221245</v>
       </c>
       <c r="Z25" t="n">
         <v>0</v>
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-2.439483664451092</v>
+        <v>1.104996748025871</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -2514,7 +2514,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>5.664332984950206</v>
+        <v>2.773264146949486</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -2532,7 +2532,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>-2.535054021863906</v>
+        <v>1.108453806498179</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
@@ -2541,7 +2541,7 @@
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>5.482191757330714</v>
+        <v>2.835582125834184</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2559,7 +2559,7 @@
         <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>5.800013154550886</v>
+        <v>3.186849911762807</v>
       </c>
       <c r="X26" t="n">
         <v>0</v>
@@ -2568,7 +2568,7 @@
         <v>0</v>
       </c>
       <c r="Z26" t="n">
-        <v>6.104390756662324</v>
+        <v>4.852972916221245</v>
       </c>
       <c r="AA26" t="n">
         <v>0</v>
@@ -2576,13 +2576,13 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-1.409831173295371</v>
+        <v>-1.082744751304861</v>
       </c>
       <c r="B27" t="n">
-        <v>-3.887214466383659</v>
+        <v>-3.146205412947956</v>
       </c>
       <c r="C27" t="n">
-        <v>-3.982228449644786</v>
+        <v>-3.398737595875454</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -2591,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8084629721561751</v>
+        <v>-0.4240457302122232</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -2600,16 +2600,16 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.9628671033800138</v>
+        <v>0.1989722918107112</v>
       </c>
       <c r="J27" t="n">
-        <v>1.40567882475756</v>
+        <v>1.082116365985503</v>
       </c>
       <c r="K27" t="n">
-        <v>3.660787614650573</v>
+        <v>3.143762882042221</v>
       </c>
       <c r="L27" t="n">
-        <v>4.283930900581249</v>
+        <v>3.399704775832141</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -2618,7 +2618,7 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>1.279939865673288</v>
+        <v>-0.4143579642504828</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2627,16 +2627,16 @@
         <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>0.4547387423596508</v>
+        <v>0.2741241008832271</v>
       </c>
       <c r="S27" t="n">
-        <v>0.05992407407311829</v>
+        <v>1.430469241323062e-17</v>
       </c>
       <c r="T27" t="n">
-        <v>0.2488233324784572</v>
+        <v>5.975038172567615e-16</v>
       </c>
       <c r="U27" t="n">
-        <v>0.4538947839540482</v>
+        <v>9.033572501149223e-16</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="X27" t="n">
-        <v>7.400257187162005</v>
+        <v>3.83372519930778</v>
       </c>
       <c r="Y27" t="n">
         <v>0</v>
@@ -2654,7 +2654,7 @@
         <v>0</v>
       </c>
       <c r="AA27" t="n">
-        <v>9.154176534540113</v>
+        <v>5.963278060818974</v>
       </c>
     </row>
   </sheetData>

</xml_diff>